<commit_message>
feat: added metrics module
</commit_message>
<xml_diff>
--- a/dataset/Validation.xlsx
+++ b/dataset/Validation.xlsx
@@ -1,31 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28110"/>
-  <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_C3DBBB911BE2B1982A9CBF3B82709A776C0CCEEE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1"/>
     </ext>
@@ -36,163 +22,183 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="54">
   <si>
-    <t>Cláusulas</t>
-  </si>
-  <si>
-    <t>Legalidad (L) Ilegalidad (I)</t>
-  </si>
-  <si>
-    <t>Abusividad (N:No; S:Sí)</t>
-  </si>
-  <si>
-    <t>Areas de Riesgo</t>
-  </si>
-  <si>
-    <t>Vaguedades</t>
-  </si>
-  <si>
-    <t>Lagunas</t>
-  </si>
-  <si>
-    <t>Obligaciones Pendientes del Inquilino</t>
-  </si>
-  <si>
-    <t>Cláusulas Adicionales</t>
-  </si>
-  <si>
-    <t>Cambios Futuros (ya están vigentes)</t>
-  </si>
-  <si>
-    <t>Objeto</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>Cambio de Titularidad de Suministros: 30 días</t>
-  </si>
-  <si>
-    <t>Inventario</t>
-  </si>
-  <si>
-    <t>Límite Incremento Renta</t>
-  </si>
-  <si>
-    <t>Plazo/Duración</t>
-  </si>
-  <si>
-    <t>I</t>
-  </si>
-  <si>
-    <t>Contratación de Seguro de Responsabilidad Civil: 30 días</t>
-  </si>
-  <si>
-    <t>Seguro Responsabilidad Civil</t>
-  </si>
-  <si>
-    <t>Zonas de Mercado Residencial Tensionado</t>
-  </si>
-  <si>
-    <t>Plazo/Desistimiento</t>
+    <t xml:space="preserve">Cláusulas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legalidad (L) Ilegalidad (I)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abusividad (N:No; S:Sí)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Areas de Riesgo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vaguedades</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lagunas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Obligaciones Pendientes del Inquilino</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cláusulas Adicionales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cambios Futuros (ya están vigentes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Objeto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cambio de Titularidad de Suministros: 30 días</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inventario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Límite Incremento Renta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plazo/Duración</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contratación de Seguro de Responsabilidad Civil: 30 días</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seguro Responsabilidad Civil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zonas de Mercado Residencial Tensionado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plazo/Desistimiento</t>
   </si>
   <si>
     <t xml:space="preserve"> Notificación de Visitas Prolongadas: 30 días</t>
   </si>
   <si>
-    <t>Políticas de Visitas</t>
-  </si>
-  <si>
-    <t>Bases de Datos de Contratos de Arrendamiento</t>
-  </si>
-  <si>
-    <t>Entrega Inmueble/Condiciones</t>
-  </si>
-  <si>
-    <t>Obligaciones Pendientes del Propietario</t>
-  </si>
-  <si>
-    <t>Cambio Titularidad de Suministros</t>
-  </si>
-  <si>
-    <t>Entrega Inmueble/Llaves</t>
+    <t xml:space="preserve">Políticas de Visitas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bases de Datos de Contratos de Arrendamiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrega Inmueble/Condiciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Obligaciones Pendientes del Propietario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cambio Titularidad de Suministros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrega Inmueble/Llaves</t>
   </si>
   <si>
     <t xml:space="preserve">Entrega del Inmueble en Buen Estado. </t>
   </si>
   <si>
-    <t>Subrogación</t>
-  </si>
-  <si>
-    <t>Renta/Monto</t>
-  </si>
-  <si>
-    <t>Mantenimiento de Servicios y Suministros</t>
-  </si>
-  <si>
-    <t>Revisión Fianza. Plazo de tres años no es correcto. Ahora es 5 años arrendador PF y y 7 años PJ.</t>
-  </si>
-  <si>
-    <t>Renta/Actualización</t>
-  </si>
-  <si>
-    <t>Mantenimiento y reparaciones.</t>
-  </si>
-  <si>
-    <t>Renta/Impago</t>
-  </si>
-  <si>
-    <t>Normas de convivencia</t>
-  </si>
-  <si>
-    <t>Garantía/Fianza</t>
-  </si>
-  <si>
-    <t>Obras de mejoras. No es correcta</t>
-  </si>
-  <si>
-    <t>Garantía/Aval</t>
-  </si>
-  <si>
-    <t>Resolución Anticipada. Hay que mejorar la redacción que ofrece ChatGPT.</t>
-  </si>
-  <si>
-    <t>Servicios/Gastos</t>
-  </si>
-  <si>
-    <t>Servicios/Interrupciones</t>
-  </si>
-  <si>
-    <t>Gatos/Reparaciones</t>
-  </si>
-  <si>
-    <t>Obras Inmueble</t>
-  </si>
-  <si>
-    <t>Devolución Inmueble/Condiciones</t>
-  </si>
-  <si>
-    <t>Devolución Inmueble/Penalización retraso</t>
-  </si>
-  <si>
-    <t>Derecho de Tanteo</t>
-  </si>
-  <si>
-    <t>Causas Terminación Contrato</t>
-  </si>
-  <si>
-    <t>Protección de Datos/Tratamiento</t>
-  </si>
-  <si>
-    <t>Protección de Datos/Cesión</t>
-  </si>
-  <si>
-    <t>Ley Aplicable</t>
+    <t xml:space="preserve">Subrogación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renta/Monto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mantenimiento de Servicios y Suministros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisión Fianza. Plazo de tres años no es correcto. Ahora es 5 años arrendador PF y y 7 años PJ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renta/Actualización</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mantenimiento y reparaciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renta/Impago</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Normas de convivencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Garantía/Fianza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Obras de mejoras. No es correcta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Garantía/Aval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resolución Anticipada. Hay que mejorar la redacción que ofrece ChatGPT.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servicios/Gastos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servicios/Interrupciones</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <u val="single"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Gastos</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/Reparaciones</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Obras Inmueble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Devolución Inmueble/Condiciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Devolución Inmueble/Penalización retraso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Derecho de Tanteo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Causas Terminación Contrato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protección de Datos/Tratamiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protección de Datos/Cesión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ley Aplicable</t>
   </si>
   <si>
     <t xml:space="preserve">Firma </t>
@@ -201,8 +207,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="General"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -210,7 +219,30 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <u val="single"/>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -226,117 +258,138 @@
     </fill>
   </fills>
   <borders count="2">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="hair">
-        <color auto="1"/>
-      </left>
-      <right style="hair">
-        <color auto="1"/>
-      </right>
-      <top style="hair">
-        <color auto="1"/>
-      </top>
-      <bottom style="hair">
-        <color auto="1"/>
-      </bottom>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="hair"/>
+      <right style="hair"/>
+      <top style="hair"/>
+      <bottom style="hair"/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+  <cellXfs count="7">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
   <a:themeElements>
     <a:clrScheme name="LibreOffice">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18A303"/>
+        <a:srgbClr val="18a303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369A3"/>
+        <a:srgbClr val="0369a3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A33E03"/>
+        <a:srgbClr val="a33e03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8E03A3"/>
+        <a:srgbClr val="8e03a3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="C99C00"/>
+        <a:srgbClr val="c99c00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="C9211E"/>
+        <a:srgbClr val="c9211e"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000EE"/>
+        <a:srgbClr val="0000ee"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551A8B"/>
+        <a:srgbClr val="551a8b"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="DejaVu Sans"/>
-        <a:cs typeface="DejaVu Sans"/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="DejaVu Sans"/>
-        <a:cs typeface="DejaVu Sans"/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -389,23 +442,24 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A3:I34"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="15.140625" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15.14"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:9" ht="34.9">
+    <row r="3" customFormat="false" ht="34.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -434,7 +488,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="46.15">
+    <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -463,7 +517,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="46.15">
+    <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -492,7 +546,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="46.15">
+    <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
@@ -521,7 +575,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="34.9">
+    <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>25</v>
       </c>
@@ -548,7 +602,7 @@
       </c>
       <c r="I7" s="3"/>
     </row>
-    <row r="8" spans="1:9" ht="34.9">
+    <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>28</v>
       </c>
@@ -575,7 +629,7 @@
       </c>
       <c r="I8" s="3"/>
     </row>
-    <row r="9" spans="1:9" ht="79.7">
+    <row r="9" customFormat="false" ht="79.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
         <v>31</v>
       </c>
@@ -602,7 +656,7 @@
       </c>
       <c r="I9" s="3"/>
     </row>
-    <row r="10" spans="1:9" ht="23.65">
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>34</v>
       </c>
@@ -627,7 +681,7 @@
       </c>
       <c r="I10" s="3"/>
     </row>
-    <row r="11" spans="1:9" ht="23.65">
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>36</v>
       </c>
@@ -652,7 +706,7 @@
       </c>
       <c r="I11" s="3"/>
     </row>
-    <row r="12" spans="1:9" ht="34.9">
+    <row r="12" customFormat="false" ht="34.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
         <v>38</v>
       </c>
@@ -677,7 +731,7 @@
       </c>
       <c r="I12" s="3"/>
     </row>
-    <row r="13" spans="1:9" ht="57.4">
+    <row r="13" customFormat="false" ht="57" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
         <v>40</v>
       </c>
@@ -702,7 +756,7 @@
       </c>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
         <v>42</v>
       </c>
@@ -725,7 +779,7 @@
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
     </row>
-    <row r="15" spans="1:9" ht="23.65">
+    <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>43</v>
       </c>
@@ -748,8 +802,8 @@
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
     </row>
-    <row r="16" spans="1:9" ht="23.65">
-      <c r="A16" s="2" t="s">
+    <row r="16" customFormat="false" ht="27.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
         <v>44</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -771,7 +825,7 @@
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" customFormat="false" ht="18.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>45</v>
       </c>
@@ -794,7 +848,7 @@
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
     </row>
-    <row r="18" spans="1:9" ht="34.9">
+    <row r="18" customFormat="false" ht="45.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
         <v>46</v>
       </c>
@@ -817,7 +871,7 @@
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
     </row>
-    <row r="19" spans="1:9" ht="34.9">
+    <row r="19" customFormat="false" ht="47.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
         <v>47</v>
       </c>
@@ -840,7 +894,7 @@
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
     </row>
-    <row r="20" spans="1:9" ht="23.65">
+    <row r="20" customFormat="false" ht="34.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
         <v>48</v>
       </c>
@@ -863,7 +917,7 @@
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
     </row>
-    <row r="21" spans="1:9" ht="34.9">
+    <row r="21" customFormat="false" ht="37.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
         <v>49</v>
       </c>
@@ -886,7 +940,7 @@
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
     </row>
-    <row r="22" spans="1:9" ht="23.65">
+    <row r="22" customFormat="false" ht="38.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
         <v>50</v>
       </c>
@@ -909,7 +963,7 @@
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
     </row>
-    <row r="23" spans="1:9" ht="23.65">
+    <row r="23" customFormat="false" ht="30.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
         <v>51</v>
       </c>
@@ -932,7 +986,7 @@
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" customFormat="false" ht="17.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
         <v>52</v>
       </c>
@@ -955,7 +1009,7 @@
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
         <v>53</v>
       </c>
@@ -978,41 +1032,42 @@
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
     </row>
-    <row r="26" spans="1:9">
-      <c r="D26" s="5"/>
-      <c r="F26" s="5"/>
-    </row>
-    <row r="27" spans="1:9">
-      <c r="D27" s="5"/>
-      <c r="F27" s="5"/>
-    </row>
-    <row r="28" spans="1:9">
-      <c r="F28" s="5"/>
-    </row>
-    <row r="29" spans="1:9">
-      <c r="F29" s="5"/>
-    </row>
-    <row r="30" spans="1:9">
-      <c r="F30" s="5"/>
-    </row>
-    <row r="31" spans="1:9">
-      <c r="F31" s="5"/>
-    </row>
-    <row r="32" spans="1:9">
-      <c r="F32" s="5"/>
-    </row>
-    <row r="33" spans="6:6">
-      <c r="F33" s="5"/>
-    </row>
-    <row r="34" spans="6:6">
-      <c r="F34" s="5"/>
+    <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D26" s="6"/>
+      <c r="F26" s="6"/>
+    </row>
+    <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D27" s="6"/>
+      <c r="F27" s="6"/>
+    </row>
+    <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F28" s="6"/>
+    </row>
+    <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F29" s="6"/>
+    </row>
+    <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F30" s="6"/>
+    </row>
+    <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F31" s="6"/>
+    </row>
+    <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F32" s="6"/>
+    </row>
+    <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F33" s="6"/>
+    </row>
+    <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F34" s="6"/>
     </row>
   </sheetData>
-  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup paperSize="9" orientation="landscape" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
-  <headerFooter>
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>